<commit_message>
Update with new dataset
</commit_message>
<xml_diff>
--- a/2026 New/Results/2026.05.06 Results_period_ols_scenarios.xlsx
+++ b/2026 New/Results/2026.05.06 Results_period_ols_scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1f12debbb769dbfe/Database/GRIP/2026 New/Results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{90D8446E-AFC0-4A49-AA7D-AD268A4DB13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED9BA3FF-A0FF-5A4C-AD3B-E9A0BE068268}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{90D8446E-AFC0-4A49-AA7D-AD268A4DB13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75ED3CA8-AA8E-FC49-A2A9-389CCC0C63CB}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20000" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Interpretation" sheetId="9" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14336" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14400" uniqueCount="917">
   <si>
     <t>scenario</t>
   </si>
@@ -2736,9 +2736,6 @@
   </si>
   <si>
     <t>ln_sales (firm size)</t>
-  </si>
-  <si>
-    <t>Mixed and unstable. Negative in P1, mildly positive in P2–P3, weaker after winsorisation</t>
   </si>
   <si>
     <t>Consistently insignificant</t>
@@ -3172,6 +3169,141 @@
   </si>
   <si>
     <t>This supports a broader conclusion that resilience is not a fixed organisational trait, but rather a dynamic outcome shaped by the interaction between organisational characteristics, sectoral structure, and changing macroeconomic conditions.</t>
+  </si>
+  <si>
+    <t>Firm size does not show a stable resilience effect. In the broader sample, size appears phase-dependent: larger firms may have been less adaptive during the initial shock but more stable during later normalisation. Inside manufacturing, size provides little differentiation.</t>
+  </si>
+  <si>
+    <t>Internationalisation is not a universal resilience advantage. Its impact changes across crisis phases and appears much weaker inside manufacturing, where firms are structurally more internationalised already.</t>
+  </si>
+  <si>
+    <t>Operational intensity behaves differently across phases. Fast asset utilisation may help during rebound periods but become a burden during stabilisation and margin compression.</t>
+  </si>
+  <si>
+    <t>Financial conservatism appears to involve trade-offs. Lower leverage may reduce early flexibility but support endurance during later phases of instability.</t>
+  </si>
+  <si>
+    <t>Productivity effects differ by population. In the broader sample, high productivity may reflect mature firms with slower expansion. In manufacturing, productivity seems more useful during rebound periods only.</t>
+  </si>
+  <si>
+    <t>Weak and insignificant throughout</t>
+  </si>
+  <si>
+    <t>Ownership structure alone provides limited explanatory power for resilience outcomes.</t>
+  </si>
+  <si>
+    <t>Internationalisation effects depend on organisational structure and crisis phase. In manufacturing, firms appear too homogeneous for the interaction to provide strong explanatory power.</t>
+  </si>
+  <si>
+    <t>Weak in P2 but strongly negative in P3</t>
+  </si>
+  <si>
+    <t>Mean reversion and cyclical correction dynamics are present in both samples, but become especially strong in the later manufacturing phase.</t>
+  </si>
+  <si>
+    <t>Sectoral exposure is one of the strongest resilience determinants. Results suggest that macroeconomic and industry-specific conditions shape outcomes more strongly than stable firm-level traits.</t>
+  </si>
+  <si>
+    <t>Manufacturing outcomes are much more influenced by extreme firms and outliers, suggesting greater sensitivity to cyclical shocks and exceptional performers.</t>
+  </si>
+  <si>
+    <t>FULL-period models</t>
+  </si>
+  <si>
+    <t>Similar weakening, though some sector effects remain strong</t>
+  </si>
+  <si>
+    <t>Several variables significant within individual phases lose explanatory power over the full 2019–2024 horizon. This suggests that many resilience drivers are temporary and regime-specific rather than stable long-term advantages.</t>
+  </si>
+  <si>
+    <t>The broader sample reflects a combination of firm-level and sectoral mechanisms, while manufacturing resilience appears more strongly shaped by changing macroeconomic regimes.</t>
+  </si>
+  <si>
+    <t>Important but unstable and highly phase-dependent</t>
+  </si>
+  <si>
+    <t>Surprisingly weak and inconsistent</t>
+  </si>
+  <si>
+    <t>Export orientation should be interpreted as a context-dependent exposure mechanism rather than a stable resilience capability.</t>
+  </si>
+  <si>
+    <t>Combination of firm characteristics, sectoral exposure, and macroeconomic timing</t>
+  </si>
+  <si>
+    <t>Sectoral and regime dynamics dominate</t>
+  </si>
+  <si>
+    <t>The results support a dynamic interpretation of resilience. Resilience does not appear to be a fixed organisational trait, but rather a shifting outcome shaped by the interaction between organisational characteristics, sector structure, and changing macroeconomic conditions.</t>
+  </si>
+  <si>
+    <t>Mostly weak in winsorised models; negative in P1 and mildly positive in P3 in raw models; neutral in FULL</t>
+  </si>
+  <si>
+    <t>Consistently insignificant in both winsorised and raw models</t>
+  </si>
+  <si>
+    <t>Positive and significant in winsorised P1–P2 and FULL; weaker than in raw models</t>
+  </si>
+  <si>
+    <t>Much weaker in winsorised models than raw models; negative in P3 winsorised</t>
+  </si>
+  <si>
+    <t>Profitability supports early adaptation and rebound capacity, but manufacturing results are strongly influenced by extreme firms. Raw models suggest stronger effects than the more conservative winsorised specification.</t>
+  </si>
+  <si>
+    <t>Mostly weak in winsorised models except strong positive P3 effect; stronger and more volatile in raw models</t>
+  </si>
+  <si>
+    <t>Weak and insignificant in both winsorised and raw models</t>
+  </si>
+  <si>
+    <t>Negative and relatively stable in winsorised models, especially P1 and FULL</t>
+  </si>
+  <si>
+    <t>Positive in P2 winsorised but strongly negative in P3 and FULL</t>
+  </si>
+  <si>
+    <t>Mostly weak in winsorised models; stronger positive effects visible in raw P3</t>
+  </si>
+  <si>
+    <t>Weak and unstable; negative in raw P1, weak elsewhere</t>
+  </si>
+  <si>
+    <t>Mildly negative in winsorised P3 and FULL; stronger negative effects in raw models</t>
+  </si>
+  <si>
+    <t>Mildly positive in winsorised P2 only; otherwise weak</t>
+  </si>
+  <si>
+    <t>Weak throughout; one negative effect in winsorised FULL</t>
+  </si>
+  <si>
+    <t>Mostly weak in winsorised models except strongly negative in P3; more volatile in raw models</t>
+  </si>
+  <si>
+    <t>Strongly negative in winsorised P2–P3</t>
+  </si>
+  <si>
+    <t>Strong throughout winsorised and raw models, with major directional shifts across periods</t>
+  </si>
+  <si>
+    <t>Very strong and often dominant in both specifications</t>
+  </si>
+  <si>
+    <t>Moderate; most core patterns remain visible though weaker</t>
+  </si>
+  <si>
+    <t>Very strong; many raw effects weaken or disappear after winsorisation</t>
+  </si>
+  <si>
+    <t>Many phase-specific effects weaken or disappear in winsorised FULL models</t>
+  </si>
+  <si>
+    <t>Winsorised models remain relatively balanced and interpretable</t>
+  </si>
+  <si>
+    <t>Winsorised models remain more cyclical and reversal-driven</t>
   </si>
 </sst>
 </file>
@@ -3563,16 +3695,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD2B71E4-D0A4-0049-817B-175913C7A1F5}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="68.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="61.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="157.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="74" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="55.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="212.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>738</v>
       </c>
@@ -3585,290 +3721,485 @@
       <c r="D1" s="2" t="s">
         <v>741</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F1" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>739</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>742</v>
       </c>
       <c r="B2" t="s">
+        <v>894</v>
+      </c>
+      <c r="C2" t="s">
         <v>743</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>744</v>
       </c>
-      <c r="D2" t="s">
-        <v>745</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F2" t="s">
+        <v>742</v>
+      </c>
+      <c r="G2" t="s">
+        <v>894</v>
+      </c>
+      <c r="H2" t="s">
+        <v>895</v>
+      </c>
+      <c r="I2" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>103</v>
       </c>
       <c r="B3" t="s">
+        <v>745</v>
+      </c>
+      <c r="C3" t="s">
         <v>746</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>747</v>
       </c>
-      <c r="D3" t="s">
-        <v>748</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3" t="s">
+        <v>896</v>
+      </c>
+      <c r="H3" t="s">
+        <v>897</v>
+      </c>
+      <c r="I3" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>104</v>
       </c>
       <c r="B4" t="s">
+        <v>748</v>
+      </c>
+      <c r="C4" t="s">
         <v>749</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>750</v>
       </c>
-      <c r="D4" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>104</v>
+      </c>
+      <c r="G4" t="s">
+        <v>899</v>
+      </c>
+      <c r="H4" t="s">
+        <v>900</v>
+      </c>
+      <c r="I4" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>105</v>
       </c>
       <c r="B5" t="s">
+        <v>751</v>
+      </c>
+      <c r="C5" t="s">
         <v>752</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>753</v>
       </c>
-      <c r="D5" t="s">
-        <v>754</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>105</v>
+      </c>
+      <c r="G5" t="s">
+        <v>901</v>
+      </c>
+      <c r="H5" t="s">
+        <v>902</v>
+      </c>
+      <c r="I5" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>106</v>
       </c>
       <c r="B6" t="s">
+        <v>754</v>
+      </c>
+      <c r="C6" t="s">
         <v>755</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>756</v>
       </c>
-      <c r="D6" t="s">
-        <v>757</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G6" t="s">
+        <v>903</v>
+      </c>
+      <c r="H6" t="s">
+        <v>904</v>
+      </c>
+      <c r="I6" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>107</v>
       </c>
       <c r="B7" t="s">
+        <v>757</v>
+      </c>
+      <c r="C7" t="s">
         <v>758</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>759</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G7" t="s">
+        <v>905</v>
+      </c>
+      <c r="H7" t="s">
+        <v>906</v>
+      </c>
+      <c r="I7" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>760</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="B8" t="s">
         <v>761</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>762</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>763</v>
       </c>
-      <c r="D8" t="s">
+      <c r="F8" t="s">
+        <v>760</v>
+      </c>
+      <c r="G8" t="s">
+        <v>907</v>
+      </c>
+      <c r="H8" t="s">
+        <v>877</v>
+      </c>
+      <c r="I8" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>764</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="B9" t="s">
         <v>765</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>766</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>767</v>
       </c>
-      <c r="D9" t="s">
+      <c r="F9" t="s">
+        <v>764</v>
+      </c>
+      <c r="G9" t="s">
+        <v>908</v>
+      </c>
+      <c r="H9" t="s">
+        <v>877</v>
+      </c>
+      <c r="I9" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>768</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="B10" t="s">
         <v>769</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>770</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>771</v>
       </c>
-      <c r="D10" t="s">
+      <c r="F10" t="s">
+        <v>768</v>
+      </c>
+      <c r="G10" t="s">
+        <v>909</v>
+      </c>
+      <c r="H10" t="s">
+        <v>880</v>
+      </c>
+      <c r="I10" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>772</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="B11" t="s">
         <v>773</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>774</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>775</v>
       </c>
-      <c r="D11" t="s">
+      <c r="F11" t="s">
+        <v>772</v>
+      </c>
+      <c r="G11" t="s">
+        <v>910</v>
+      </c>
+      <c r="H11" t="s">
+        <v>911</v>
+      </c>
+      <c r="I11" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>776</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="B12" t="s">
         <v>777</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>774</v>
+      </c>
+      <c r="D12" t="s">
         <v>778</v>
       </c>
-      <c r="C12" t="s">
-        <v>775</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="F12" t="s">
+        <v>776</v>
+      </c>
+      <c r="G12" t="s">
+        <v>912</v>
+      </c>
+      <c r="H12" t="s">
+        <v>913</v>
+      </c>
+      <c r="I12" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>779</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="B13" t="s">
         <v>780</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>781</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>782</v>
       </c>
-      <c r="D13" t="s">
+      <c r="F13" t="s">
+        <v>884</v>
+      </c>
+      <c r="G13" t="s">
+        <v>914</v>
+      </c>
+      <c r="H13" t="s">
+        <v>885</v>
+      </c>
+      <c r="I13" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>783</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+      <c r="B14" t="s">
         <v>784</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>785</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>786</v>
       </c>
-      <c r="D14" t="s">
+      <c r="F14" t="s">
+        <v>779</v>
+      </c>
+      <c r="G14" t="s">
+        <v>915</v>
+      </c>
+      <c r="H14" t="s">
+        <v>916</v>
+      </c>
+      <c r="I14" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>787</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="B15" t="s">
         <v>788</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>789</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>790</v>
       </c>
-      <c r="D15" t="s">
-        <v>791</v>
+      <c r="F15" t="s">
+        <v>783</v>
+      </c>
+      <c r="G15" t="s">
+        <v>888</v>
+      </c>
+      <c r="H15" t="s">
+        <v>889</v>
+      </c>
+      <c r="I15" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>787</v>
+      </c>
+      <c r="G16" t="s">
+        <v>891</v>
+      </c>
+      <c r="H16" t="s">
+        <v>892</v>
+      </c>
+      <c r="I16" t="s">
+        <v>893</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -4383,157 +4714,157 @@
     </row>
     <row r="24" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="56" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="57" spans="1:1" ht="19" x14ac:dyDescent="0.25">
@@ -4541,167 +4872,167 @@
     </row>
     <row r="58" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="62" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="68" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="77" spans="1:1" ht="19" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
   </sheetData>

</xml_diff>